<commit_message>
correction derive reg entropique
</commit_message>
<xml_diff>
--- a/CardamomOT_inputs.xlsx
+++ b/CardamomOT_inputs.xlsx
@@ -1087,7 +1087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1856,67 +1856,55 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>report_net_index</t>
+          <t>report_normalize</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>report: network shown when n_networks &gt; 1</t>
+          <t>report UMAPs: counts normalised per cell</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>report_normalize</t>
+          <t>report_log1p</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>report UMAPs: counts normalised per cell</t>
+          <t>report UMAPs: log1p of the counts</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>report_log1p</t>
+          <t>report_n_umap</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>report UMAPs: log1p of the counts</t>
+          <t>report: maximal number of cells per stage in the UMAPs (0 = all)</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>report_n_umap</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>report: maximal number of cells per stage in the UMAPs (0 = all)</t>
-        </is>
-      </c>
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>Reproducibility</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="n"/>
+      <c r="C69" s="6" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="5" t="inlineStr">
-        <is>
-          <t>Reproducibility</t>
-        </is>
-      </c>
-      <c r="B70" s="6" t="n"/>
-      <c r="C70" s="6" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A70" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>Random seed for reproducibility (main process and parallel workers); None = not seeded (runs vary)</t>
         </is>

</xml_diff>

<commit_message>
extension multiple network conditions
</commit_message>
<xml_diff>
--- a/CardamomOT_inputs.xlsx
+++ b/CardamomOT_inputs.xlsx
@@ -455,6 +455,11 @@
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <t>Timepoints of the simulations (0 added if absent)</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Timepoints of the test cells (split = train; 0 added if absent): times beyond the inference ones are held out for the test only; empty = the inference timepoints</t>
       </text>
     </comment>
   </commentList>
@@ -2216,11 +2221,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2232,6 +2238,11 @@
       <c r="B1" s="4" t="inlineStr">
         <is>
           <t>times_simulation</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>times_test</t>
         </is>
       </c>
     </row>

</xml_diff>